<commit_message>
feat: fill in phone numbers for Indu Kumari and Mamta Kumari
Owner supplied both numbers directly. Indu Kumari (Accountant, role
maps to VALID_ROLES) also gets a login now that she has a real phone;
Mamta Kumari (Office Incharge, no role mapping) just gets her phone
updated, consistent with the original import.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/School_docs/Daffodils/STAFF INFO.xlsx
+++ b/School_docs/Daffodils/STAFF INFO.xlsx
@@ -1193,6 +1193,11 @@
           <t>KUMARI</t>
         </is>
       </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>6203757534</t>
+        </is>
+      </c>
       <c r="D21" t="inlineStr">
         <is>
           <t>OFFICE INCHARGE</t>
@@ -1213,6 +1218,11 @@
       <c r="B22" t="inlineStr">
         <is>
           <t>KUMARI</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>9304091054</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">

</xml_diff>